<commit_message>
added total portfolio P/L
</commit_message>
<xml_diff>
--- a/stock_tracker.xlsx
+++ b/stock_tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,10 +448,10 @@
         <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>278.45</v>
+        <v>277.83</v>
       </c>
       <c r="D2" t="n">
-        <v>178.45</v>
+        <v>177.83</v>
       </c>
     </row>
     <row r="3">
@@ -464,10 +464,10 @@
         <v>3000</v>
       </c>
       <c r="C3" t="n">
-        <v>343.06</v>
+        <v>343.92</v>
       </c>
       <c r="D3" t="n">
-        <v>-2656.94</v>
+        <v>-2656.08</v>
       </c>
     </row>
     <row r="4">
@@ -480,10 +480,10 @@
         <v>700</v>
       </c>
       <c r="C4" t="n">
-        <v>386.76</v>
+        <v>386.73</v>
       </c>
       <c r="D4" t="n">
-        <v>-313.24</v>
+        <v>-313.27</v>
       </c>
     </row>
     <row r="5">
@@ -496,10 +496,10 @@
         <v>300</v>
       </c>
       <c r="C5" t="n">
-        <v>232.32</v>
+        <v>231.8</v>
       </c>
       <c r="D5" t="n">
-        <v>-67.68000000000001</v>
+        <v>-68.2</v>
       </c>
     </row>
     <row r="6">
@@ -512,10 +512,10 @@
         <v>250</v>
       </c>
       <c r="C6" t="n">
-        <v>371.09</v>
+        <v>370.27</v>
       </c>
       <c r="D6" t="n">
-        <v>121.09</v>
+        <v>120.27</v>
       </c>
     </row>
     <row r="7">
@@ -528,10 +528,38 @@
         <v>150</v>
       </c>
       <c r="C7" t="n">
-        <v>41.19</v>
+        <v>41.15</v>
       </c>
       <c r="D7" t="n">
-        <v>-108.81</v>
+        <v>-108.85</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>350</v>
+      </c>
+      <c r="C8" t="n">
+        <v>555.59</v>
+      </c>
+      <c r="D8" t="n">
+        <v>205.59</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>-2642.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a seperate input file for stocks and buy prices
</commit_message>
<xml_diff>
--- a/stock_tracker.xlsx
+++ b/stock_tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C5" t="n">
         <v>232.69</v>
       </c>
       <c r="D5" t="n">
-        <v>-67.31</v>
+        <v>32.69</v>
       </c>
     </row>
     <row r="6">
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>250</v>
+        <v>550</v>
       </c>
       <c r="C6" t="n">
         <v>372.97</v>
       </c>
       <c r="D6" t="n">
-        <v>122.97</v>
+        <v>-177.03</v>
       </c>
     </row>
     <row r="7">
@@ -537,13 +537,29 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>300</v>
+      </c>
+      <c r="C8" t="n">
+        <v>550.25</v>
+      </c>
+      <c r="D8" t="n">
+        <v>250.25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="n">
-        <v>-2852.71</v>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>-2802.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>